<commit_message>
Evolução do REDFM / Publisher 2.3.4
</commit_message>
<xml_diff>
--- a/docs/StructureDefinition-br-core-practitionerrole.xlsx
+++ b/docs/StructureDefinition-br-core-practitionerrole.xlsx
@@ -57,7 +57,7 @@
     <t>Date</t>
   </si>
   <si>
-    <t>2026-06-30T10:02:10-03:00</t>
+    <t>2026-09-25T17:16:20-03:00</t>
   </si>
   <si>
     <t>Publisher</t>
@@ -81,7 +81,7 @@
     <t>Description</t>
   </si>
   <si>
-    <t>Este perfil restringe o recurso [PractitionerRole](https://hl7.org/fhir/R4/practitionerrole.html) que representa um conjunto específico de funções/locais/especialidades/serviços que um profissional pode desempenhar em uma organização por um período de tempo.</t>
+    <t>Este perfil restringe o recurso PractitionerRole que representa um conjunto específico de funções/locais/especialidades/serviços que um profissional pode desempenhar em uma organização por um período de tempo.</t>
   </si>
   <si>
     <t>Purpose</t>

</xml_diff>